<commit_message>
Update Fidelity outcomes and Barclays assessment status
</commit_message>
<xml_diff>
--- a/job_application_dashboard_2026-09-24.xlsx
+++ b/job_application_dashboard_2026-09-24.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R553275dbe94745f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="2" r:id="R1c7daccaee6a4b3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5669b74fb3f340ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="2" r:id="R7b38526d99f34f35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -182,7 +182,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="45">
+  <x:cellXfs count="44">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -236,9 +236,6 @@
     <x:xf numFmtId="200" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
@@ -318,7 +315,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="6">
+  <x:dxfs count="10">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -355,6 +352,28 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C2F00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF9C2F00"/>
       </x:font>
       <x:fill>
@@ -382,6 +401,28 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C2F00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -680,13 +721,13 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="E6" s="14" t="str">
-        <x:v>Assessment outstanding</x:v>
+        <x:v>OA outstanding</x:v>
       </x:c>
       <x:c r="F6" s="14" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="G6" s="14" t="str">
         <x:v>Latest submission</x:v>
-      </x:c>
-      <x:c r="G6" s="14" t="str">
-        <x:v>Source coverage</x:v>
       </x:c>
       <x:c r="H6" s="15" t="str">
         <x:v>Public resume links</x:v>
@@ -698,32 +739,33 @@
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="16" t="n">
         <x:f>COUNTA(Applications!A6:A50)</x:f>
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B7" s="17" t="n">
         <x:f>COUNTIFS(Applications!D6:D50,"Submitted")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C7" s="17" t="n">
-        <x:f>COUNTIFS(Applications!D6:D50,"Received")+COUNTIFS(Applications!D6:D50,"Received / under review")+COUNTIFS(Applications!D6:D50,"Application received")+COUNTIFS(Applications!D6:D50,"Application received / reviewing")</x:f>
-        <x:v>4</x:v>
+        <x:f>COUNTIFS(Applications!D6:D50,"Received")+COUNTIFS(Applications!D6:D50,"Received / under review")+COUNTIFS(Applications!D6:D50,"Application received / reviewing")</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D7" s="17" t="n">
         <x:f>COUNTIFS(Applications!D6:D50,"In Progress")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E7" s="17" t="n">
-        <x:f>COUNTIFS(Applications!D6:D50,"Assessment outstanding")</x:f>
+        <x:f>COUNTIFS(Applications!D6:D50,"OA outstanding")</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F7" s="18" t="n">
+      <x:c r="F7" s="17" t="n">
+        <x:f>COUNTIFS(Applications!D6:D50,"Rejected")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G7" s="18" t="n">
         <x:f>MAX(Applications!C6:C50)</x:f>
         <x:v>46289</x:v>
       </x:c>
-      <x:c r="G7" s="19" t="str">
-        <x:v>Application logs, candidate portals, and confirmation emails</x:v>
-      </x:c>
-      <x:c r="H7" s="20" t="str">
+      <x:c r="H7" s="19" t="str">
         <x:v>Click Open PDF in the tracker</x:v>
       </x:c>
       <x:c r="I7" s="2"/>
@@ -731,8 +773,8 @@
       <x:c r="K7" s="2"/>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="21" t="str">
-        <x:v>Note: Fidelity Fixed Income and Barclays are excluded because a completed submission was not verified. Balbec appears twice because two confirmed submission channels were recorded.</x:v>
+      <x:c r="A8" s="20" t="str">
+        <x:v>Evidence combines application logs, candidate portals, confirmation emails, and user-reported outcomes. Balbec appears twice because two confirmed submission channels were recorded.</x:v>
       </x:c>
       <x:c r="B8" s="2"/>
       <x:c r="C8" s="2"/>
@@ -759,22 +801,22 @@
       <x:c r="K9" s="2"/>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
-      <x:c r="A10" s="35" t="str">
+      <x:c r="A10" s="34" t="str">
         <x:v>Company</x:v>
       </x:c>
-      <x:c r="B10" s="36" t="str">
+      <x:c r="B10" s="35" t="str">
         <x:v>Role</x:v>
       </x:c>
-      <x:c r="C10" s="36" t="str">
+      <x:c r="C10" s="35" t="str">
         <x:v>Submitted</x:v>
       </x:c>
-      <x:c r="D10" s="36" t="str">
+      <x:c r="D10" s="35" t="str">
         <x:v>Current status</x:v>
       </x:c>
-      <x:c r="E10" s="36" t="str">
+      <x:c r="E10" s="35" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="F10" s="37" t="str">
+      <x:c r="F10" s="36" t="str">
         <x:v>Resume</x:v>
       </x:c>
       <x:c r="G10" s="2"/>
@@ -784,7 +826,7 @@
       <x:c r="K10" s="2"/>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
-      <x:c r="A11" s="38" t="str">
+      <x:c r="A11" s="37" t="str">
         <x:f>Applications!A6</x:f>
         <x:v>Arrowstreet Capital</x:v>
       </x:c>
@@ -792,7 +834,7 @@
         <x:f>Applications!B6</x:f>
         <x:v>Quantitative Developer Intern, Summer 2027 (R1506)</x:v>
       </x:c>
-      <x:c r="C11" s="39" t="n">
+      <x:c r="C11" s="38" t="n">
         <x:f>Applications!C6</x:f>
         <x:v>46279</x:v>
       </x:c>
@@ -804,7 +846,7 @@
         <x:f>Applications!E6</x:f>
         <x:v>Official candidate home</x:v>
       </x:c>
-      <x:c r="F11" s="40" t="e">
+      <x:c r="F11" s="39" t="e">
         <x:f>Applications!F6</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Arrowstreet_Quant_Developer_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -815,7 +857,7 @@
       <x:c r="K11" s="2"/>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
-      <x:c r="A12" s="38" t="str">
+      <x:c r="A12" s="37" t="str">
         <x:f>Applications!A7</x:f>
         <x:v>Applied Academics LLC</x:v>
       </x:c>
@@ -823,7 +865,7 @@
         <x:f>Applications!B7</x:f>
         <x:v>Quantitative Analyst Intern</x:v>
       </x:c>
-      <x:c r="C12" s="39" t="n">
+      <x:c r="C12" s="38" t="n">
         <x:f>Applications!C7</x:f>
         <x:v>46279</x:v>
       </x:c>
@@ -835,7 +877,7 @@
         <x:f>Applications!E7</x:f>
         <x:v>Handshake confirmation</x:v>
       </x:c>
-      <x:c r="F12" s="40" t="e">
+      <x:c r="F12" s="39" t="e">
         <x:f>Applications!F7</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Applied_Academics_Analyst_Intern_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -846,7 +888,7 @@
       <x:c r="K12" s="2"/>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
-      <x:c r="A13" s="38" t="str">
+      <x:c r="A13" s="37" t="str">
         <x:f>Applications!A8</x:f>
         <x:v>IMC</x:v>
       </x:c>
@@ -854,7 +896,7 @@
         <x:f>Applications!B8</x:f>
         <x:v>Quantitative Trader Intern, Summer 2027 (Chicago)</x:v>
       </x:c>
-      <x:c r="C13" s="39" t="n">
+      <x:c r="C13" s="38" t="n">
         <x:f>Applications!C8</x:f>
         <x:v>46279</x:v>
       </x:c>
@@ -866,7 +908,7 @@
         <x:f>Applications!E8</x:f>
         <x:v>Official confirmation page</x:v>
       </x:c>
-      <x:c r="F13" s="40" t="e">
+      <x:c r="F13" s="39" t="e">
         <x:f>Applications!F8</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.IMC_Trader_Intern_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -877,7 +919,7 @@
       <x:c r="K13" s="2"/>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
-      <x:c r="A14" s="38" t="str">
+      <x:c r="A14" s="37" t="str">
         <x:f>Applications!A9</x:f>
         <x:v>Balbec Capital LP</x:v>
       </x:c>
@@ -885,7 +927,7 @@
         <x:f>Applications!B9</x:f>
         <x:v>2027 Quantitative Summer Analyst</x:v>
       </x:c>
-      <x:c r="C14" s="39" t="n">
+      <x:c r="C14" s="38" t="n">
         <x:f>Applications!C9</x:f>
         <x:v>46279</x:v>
       </x:c>
@@ -897,7 +939,7 @@
         <x:f>Applications!E9</x:f>
         <x:v>Handshake confirmation</x:v>
       </x:c>
-      <x:c r="F14" s="40" t="e">
+      <x:c r="F14" s="39" t="e">
         <x:f>Applications!F9</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Summer_Analyst_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -908,7 +950,7 @@
       <x:c r="K14" s="2"/>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
-      <x:c r="A15" s="38" t="str">
+      <x:c r="A15" s="37" t="str">
         <x:f>Applications!A10</x:f>
         <x:v>Walleye Capital</x:v>
       </x:c>
@@ -916,7 +958,7 @@
         <x:f>Applications!B10</x:f>
         <x:v>Quantitative Developer Intern, Summer 2027</x:v>
       </x:c>
-      <x:c r="C15" s="39" t="n">
+      <x:c r="C15" s="38" t="n">
         <x:f>Applications!C10</x:f>
         <x:v>46279</x:v>
       </x:c>
@@ -928,7 +970,7 @@
         <x:f>Applications!E10</x:f>
         <x:v>Official confirmation page</x:v>
       </x:c>
-      <x:c r="F15" s="40" t="e">
+      <x:c r="F15" s="39" t="e">
         <x:f>Applications!F10</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Walleye_Quantic_Developer_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -939,7 +981,7 @@
       <x:c r="K15" s="2"/>
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
-      <x:c r="A16" s="38" t="str">
+      <x:c r="A16" s="37" t="str">
         <x:f>Applications!A11</x:f>
         <x:v>Seven Research</x:v>
       </x:c>
@@ -947,7 +989,7 @@
         <x:f>Applications!B11</x:f>
         <x:v>Quantitative Researcher Intern</x:v>
       </x:c>
-      <x:c r="C16" s="39" t="n">
+      <x:c r="C16" s="38" t="n">
         <x:f>Applications!C11</x:f>
         <x:v>46279</x:v>
       </x:c>
@@ -959,7 +1001,7 @@
         <x:f>Applications!E11</x:f>
         <x:v>Official confirmation page</x:v>
       </x:c>
-      <x:c r="F16" s="40" t="e">
+      <x:c r="F16" s="39" t="e">
         <x:f>Applications!F11</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Seven_Research_Quant_Researcher_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -970,7 +1012,7 @@
       <x:c r="K16" s="2"/>
     </x:row>
     <x:row r="17" ht="20" customHeight="1">
-      <x:c r="A17" s="38" t="str">
+      <x:c r="A17" s="37" t="str">
         <x:f>Applications!A12</x:f>
         <x:v>Bank of America</x:v>
       </x:c>
@@ -978,19 +1020,19 @@
         <x:f>Applications!B12</x:f>
         <x:v>Global Quantitative Research Summer Associate Program, 2027</x:v>
       </x:c>
-      <x:c r="C17" s="39" t="n">
+      <x:c r="C17" s="38" t="n">
         <x:f>Applications!C12</x:f>
         <x:v>46279</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
         <x:f>Applications!D12</x:f>
-        <x:v>Assessment outstanding</x:v>
+        <x:v>OA outstanding</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
         <x:f>Applications!E12</x:f>
         <x:v>Application Center</x:v>
       </x:c>
-      <x:c r="F17" s="40" t="e">
+      <x:c r="F17" s="39" t="e">
         <x:f>Applications!F12</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.BofA_Global_Quant_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -1001,7 +1043,7 @@
       <x:c r="K17" s="2"/>
     </x:row>
     <x:row r="18" ht="20" customHeight="1">
-      <x:c r="A18" s="38" t="str">
+      <x:c r="A18" s="37" t="str">
         <x:f>Applications!A13</x:f>
         <x:v>Fidelity Investments</x:v>
       </x:c>
@@ -1009,19 +1051,19 @@
         <x:f>Applications!B13</x:f>
         <x:v>Quantitative Research Intern, Multi-Asset Systematic Research Team</x:v>
       </x:c>
-      <x:c r="C18" s="39" t="n">
+      <x:c r="C18" s="38" t="n">
         <x:f>Applications!C13</x:f>
         <x:v>46287</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
         <x:f>Applications!D13</x:f>
-        <x:v>Application received</x:v>
+        <x:v>Rejected</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
         <x:f>Applications!E13</x:f>
-        <x:v>Workday Candidate Home</x:v>
-      </x:c>
-      <x:c r="F18" s="40" t="e">
+        <x:v>User-reported outcome</x:v>
+      </x:c>
+      <x:c r="F18" s="39" t="e">
         <x:f>Applications!F13</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Multi_Asset_Systematic_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -1032,29 +1074,29 @@
       <x:c r="K18" s="2"/>
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
-      <x:c r="A19" s="41" t="str">
+      <x:c r="A19" s="37" t="str">
         <x:f>Applications!A14</x:f>
-        <x:v>Balbec Capital LP</x:v>
-      </x:c>
-      <x:c r="B19" s="42" t="str">
+        <x:v>Fidelity Investments</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
         <x:f>Applications!B14</x:f>
-        <x:v>2027 Quantitative Summer Analyst</x:v>
-      </x:c>
-      <x:c r="C19" s="43" t="n">
+        <x:v>Quantitative Research Intern, Fixed Income Team</x:v>
+      </x:c>
+      <x:c r="C19" s="38" t="n">
         <x:f>Applications!C14</x:f>
-        <x:v>46289</x:v>
-      </x:c>
-      <x:c r="D19" s="42" t="str">
+        <x:v>46287</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="str">
         <x:f>Applications!D14</x:f>
-        <x:v>Application received / reviewing</x:v>
-      </x:c>
-      <x:c r="E19" s="42" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="str">
         <x:f>Applications!E14</x:f>
-        <x:v>Direct-portal confirmation email</x:v>
-      </x:c>
-      <x:c r="F19" s="44" t="e">
+        <x:v>User-reported outcome</x:v>
+      </x:c>
+      <x:c r="F19" s="39" t="e">
         <x:f>Applications!F14</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Quantitative_Summer_Analyst.pdf, friendlyName=Open PDF</x:v>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Fixed_Income_Quantitative_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
       <x:c r="G19" s="2"/>
       <x:c r="H19" s="2"/>
@@ -1063,12 +1105,30 @@
       <x:c r="K19" s="2"/>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
-      <x:c r="A20" s="2"/>
-      <x:c r="B20" s="2"/>
-      <x:c r="C20" s="2"/>
-      <x:c r="D20" s="2"/>
-      <x:c r="E20" s="2"/>
-      <x:c r="F20" s="2"/>
+      <x:c r="A20" s="37" t="str">
+        <x:f>Applications!A15</x:f>
+        <x:v>Barclays</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:f>Applications!B15</x:f>
+        <x:v>Quantitative Finance Associate Summer Internship Program, 2027 (New York)</x:v>
+      </x:c>
+      <x:c r="C20" s="38" t="n">
+        <x:f>Applications!C15</x:f>
+        <x:v>46288</x:v>
+      </x:c>
+      <x:c r="D20" s="12" t="str">
+        <x:f>Applications!D15</x:f>
+        <x:v>OA received</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="str">
+        <x:f>Applications!E15</x:f>
+        <x:v>User-reported OA</x:v>
+      </x:c>
+      <x:c r="F20" s="39" t="e">
+        <x:f>Applications!F15</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Barclays_Quantitative_Analytics_2027.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
       <x:c r="G20" s="2"/>
       <x:c r="H20" s="2"/>
       <x:c r="I20" s="2"/>
@@ -1076,12 +1136,30 @@
       <x:c r="K20" s="2"/>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
-      <x:c r="D21" s="2"/>
-      <x:c r="E21" s="2"/>
-      <x:c r="F21" s="2"/>
+      <x:c r="A21" s="40" t="str">
+        <x:f>Applications!A16</x:f>
+        <x:v>Balbec Capital LP</x:v>
+      </x:c>
+      <x:c r="B21" s="41" t="str">
+        <x:f>Applications!B16</x:f>
+        <x:v>2027 Quantitative Summer Analyst</x:v>
+      </x:c>
+      <x:c r="C21" s="42" t="n">
+        <x:f>Applications!C16</x:f>
+        <x:v>46289</x:v>
+      </x:c>
+      <x:c r="D21" s="41" t="str">
+        <x:f>Applications!D16</x:f>
+        <x:v>Application received / reviewing</x:v>
+      </x:c>
+      <x:c r="E21" s="41" t="str">
+        <x:f>Applications!E16</x:f>
+        <x:v>Direct-portal confirmation email</x:v>
+      </x:c>
+      <x:c r="F21" s="43" t="e">
+        <x:f>Applications!F16</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Quantitative_Summer_Analyst.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
       <x:c r="G21" s="2"/>
       <x:c r="H21" s="2"/>
       <x:c r="I21" s="2"/>
@@ -1115,9 +1193,7 @@
       <x:c r="K23" s="2"/>
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
-      <x:c r="A24" s="21" t="str">
-        <x:v>Definitions: “Submitted” is a completed application. “Received / reviewing” is an employer acknowledgment. “Assessment outstanding” means the application needs the employer’s assessment to progress.</x:v>
-      </x:c>
+      <x:c r="A24"/>
       <x:c r="B24" s="2"/>
       <x:c r="C24" s="2"/>
       <x:c r="D24" s="2"/>
@@ -1142,8 +1218,10 @@
       <x:c r="J25" s="2"/>
       <x:c r="K25" s="2"/>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="2"/>
+    <x:row r="26" ht="26" customHeight="1">
+      <x:c r="A26" s="20" t="str">
+        <x:v>Definitions: “Submitted” is a completed application. “Received / reviewing” is an employer acknowledgment. “OA outstanding” means an online assessment remains to be completed. “OA received” means the assessment invitation has been received.</x:v>
+      </x:c>
       <x:c r="B26" s="2"/>
       <x:c r="C26" s="2"/>
       <x:c r="D26" s="2"/>
@@ -1862,12 +1940,14 @@
     <x:mergeCell ref="A2:H2"/>
     <x:mergeCell ref="A3:H3"/>
     <x:mergeCell ref="A8:H8"/>
-    <x:mergeCell ref="A24:H24"/>
+    <x:mergeCell ref="A26:H26"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D11:D19">
+  <x:conditionalFormatting sqref="D11:D21">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Assessment"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="received"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Submitted"/>
+    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="OA"/>
+    <x:cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="Rejected"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1946,25 +2026,25 @@
       <x:c r="K4" s="2"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="35" t="str">
+      <x:c r="A5" s="34" t="str">
         <x:v>Company</x:v>
       </x:c>
-      <x:c r="B5" s="36" t="str">
+      <x:c r="B5" s="35" t="str">
         <x:v>Role</x:v>
       </x:c>
-      <x:c r="C5" s="36" t="str">
+      <x:c r="C5" s="35" t="str">
         <x:v>Application date</x:v>
       </x:c>
-      <x:c r="D5" s="36" t="str">
+      <x:c r="D5" s="35" t="str">
         <x:v>Current status</x:v>
       </x:c>
-      <x:c r="E5" s="36" t="str">
+      <x:c r="E5" s="35" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="F5" s="36" t="str">
+      <x:c r="F5" s="35" t="str">
         <x:v>Resume PDF</x:v>
       </x:c>
-      <x:c r="G5" s="37" t="str">
+      <x:c r="G5" s="36" t="str">
         <x:v>Notes</x:v>
       </x:c>
       <x:c r="H5" s="2"/>
@@ -1973,13 +2053,13 @@
       <x:c r="K5" s="2"/>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="38" t="str">
+      <x:c r="A6" s="37" t="str">
         <x:v>Arrowstreet Capital</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
         <x:v>Quantitative Developer Intern, Summer 2027 (R1506)</x:v>
       </x:c>
-      <x:c r="C6" s="39" t="n">
+      <x:c r="C6" s="38" t="n">
         <x:v>46279</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
@@ -1992,20 +2072,20 @@
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Arrowstreet_Quant_Developer_Intern.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Arrowstreet_Quant_Developer_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G6" s="40" t="str"/>
+      <x:c r="G6" s="39" t="str"/>
       <x:c r="H6" s="2"/>
       <x:c r="I6" s="2"/>
       <x:c r="J6" s="2"/>
       <x:c r="K6" s="2"/>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="38" t="str">
+      <x:c r="A7" s="37" t="str">
         <x:v>Applied Academics LLC</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
         <x:v>Quantitative Analyst Intern</x:v>
       </x:c>
-      <x:c r="C7" s="39" t="n">
+      <x:c r="C7" s="38" t="n">
         <x:v>46279</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
@@ -2018,20 +2098,20 @@
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Applied_Academics_Analyst_Intern_JD.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Applied_Academics_Analyst_Intern_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G7" s="40" t="str"/>
+      <x:c r="G7" s="39" t="str"/>
       <x:c r="H7" s="2"/>
       <x:c r="I7" s="2"/>
       <x:c r="J7" s="2"/>
       <x:c r="K7" s="2"/>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="38" t="str">
+      <x:c r="A8" s="37" t="str">
         <x:v>IMC</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
         <x:v>Quantitative Trader Intern, Summer 2027 (Chicago)</x:v>
       </x:c>
-      <x:c r="C8" s="39" t="n">
+      <x:c r="C8" s="38" t="n">
         <x:v>46279</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
@@ -2044,20 +2124,20 @@
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.IMC_Trader_Intern_JD.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.IMC_Trader_Intern_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G8" s="40" t="str"/>
+      <x:c r="G8" s="39" t="str"/>
       <x:c r="H8" s="2"/>
       <x:c r="I8" s="2"/>
       <x:c r="J8" s="2"/>
       <x:c r="K8" s="2"/>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="38" t="str">
+      <x:c r="A9" s="37" t="str">
         <x:v>Balbec Capital LP</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
         <x:v>2027 Quantitative Summer Analyst</x:v>
       </x:c>
-      <x:c r="C9" s="39" t="n">
+      <x:c r="C9" s="38" t="n">
         <x:v>46279</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
@@ -2070,20 +2150,20 @@
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Summer_Analyst_JD.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Summer_Analyst_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G9" s="40" t="str"/>
+      <x:c r="G9" s="39" t="str"/>
       <x:c r="H9" s="2"/>
       <x:c r="I9" s="2"/>
       <x:c r="J9" s="2"/>
       <x:c r="K9" s="2"/>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="38" t="str">
+      <x:c r="A10" s="37" t="str">
         <x:v>Walleye Capital</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
         <x:v>Quantitative Developer Intern, Summer 2027</x:v>
       </x:c>
-      <x:c r="C10" s="39" t="n">
+      <x:c r="C10" s="38" t="n">
         <x:v>46279</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
@@ -2096,20 +2176,20 @@
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Walleye_Quantic_Developer_Intern.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Walleye_Quantic_Developer_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G10" s="40" t="str"/>
+      <x:c r="G10" s="39" t="str"/>
       <x:c r="H10" s="2"/>
       <x:c r="I10" s="2"/>
       <x:c r="J10" s="2"/>
       <x:c r="K10" s="2"/>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="38" t="str">
+      <x:c r="A11" s="37" t="str">
         <x:v>Seven Research</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
         <x:v>Quantitative Researcher Intern</x:v>
       </x:c>
-      <x:c r="C11" s="39" t="n">
+      <x:c r="C11" s="38" t="n">
         <x:v>46279</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
@@ -2122,24 +2202,24 @@
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Seven_Research_Quant_Researcher_Intern.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Seven_Research_Quant_Researcher_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G11" s="40" t="str"/>
+      <x:c r="G11" s="39" t="str"/>
       <x:c r="H11" s="2"/>
       <x:c r="I11" s="2"/>
       <x:c r="J11" s="2"/>
       <x:c r="K11" s="2"/>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
-      <x:c r="A12" s="38" t="str">
+      <x:c r="A12" s="37" t="str">
         <x:v>Bank of America</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
         <x:v>Global Quantitative Research Summer Associate Program, 2027</x:v>
       </x:c>
-      <x:c r="C12" s="39" t="n">
+      <x:c r="C12" s="38" t="n">
         <x:v>46279</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>Assessment outstanding</x:v>
+        <x:v>OA outstanding</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
         <x:v>Application Center</x:v>
@@ -2148,8 +2228,8 @@
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.BofA_Global_Quant_Research_2027.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.BofA_Global_Quant_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G12" s="40" t="str">
-        <x:v>Application submitted; employer assessment is still required.</x:v>
+      <x:c r="G12" s="39" t="str">
+        <x:v>Application submitted; the employer's online assessment is still required.</x:v>
       </x:c>
       <x:c r="H12" s="2"/>
       <x:c r="I12" s="2"/>
@@ -2157,78 +2237,110 @@
       <x:c r="K12" s="2"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="38" t="str">
+      <x:c r="A13" s="37" t="str">
         <x:v>Fidelity Investments</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
         <x:v>Quantitative Research Intern, Multi-Asset Systematic Research Team</x:v>
       </x:c>
-      <x:c r="C13" s="39" t="n">
+      <x:c r="C13" s="38" t="n">
         <x:v>46287</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>Application received</x:v>
+        <x:v>Rejected</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>Workday Candidate Home</x:v>
+        <x:v>User-reported outcome</x:v>
       </x:c>
       <x:c r="F13" s="12" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Multi_Asset_Systematic_Research_2027.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Multi_Asset_Systematic_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G13" s="40" t="str"/>
+      <x:c r="G13" s="39" t="str">
+        <x:v>Application outcome reported as rejected.</x:v>
+      </x:c>
       <x:c r="H13" s="2"/>
       <x:c r="I13" s="2"/>
       <x:c r="J13" s="2"/>
       <x:c r="K13" s="2"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="41" t="str">
-        <x:v>Balbec Capital LP</x:v>
-      </x:c>
-      <x:c r="B14" s="42" t="str">
-        <x:v>2027 Quantitative Summer Analyst</x:v>
-      </x:c>
-      <x:c r="C14" s="43" t="n">
-        <x:v>46289</x:v>
-      </x:c>
-      <x:c r="D14" s="42" t="str">
-        <x:v>Application received / reviewing</x:v>
-      </x:c>
-      <x:c r="E14" s="42" t="str">
-        <x:v>Direct-portal confirmation email</x:v>
-      </x:c>
-      <x:c r="F14" s="42" t="e">
-        <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Quantitative_Summer_Analyst.pdf","Open PDF")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Quantitative_Summer_Analyst.pdf, friendlyName=Open PDF</x:v>
-      </x:c>
-      <x:c r="G14" s="44" t="str"/>
+      <x:c r="A14" s="37" t="str">
+        <x:v>Fidelity Investments</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>Quantitative Research Intern, Fixed Income Team</x:v>
+      </x:c>
+      <x:c r="C14" s="38" t="n">
+        <x:v>46287</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="str">
+        <x:v>User-reported outcome</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="e">
+        <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Fixed_Income_Quantitative_Research_2027.pdf","Open PDF")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Fixed_Income_Quantitative_Research_2027.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
+      <x:c r="G14" s="39" t="str">
+        <x:v>Application outcome reported as rejected.</x:v>
+      </x:c>
       <x:c r="H14" s="2"/>
       <x:c r="I14" s="2"/>
       <x:c r="J14" s="2"/>
       <x:c r="K14" s="2"/>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="2"/>
-      <x:c r="B15" s="2"/>
-      <x:c r="C15" s="2"/>
-      <x:c r="D15" s="2"/>
-      <x:c r="E15" s="2"/>
-      <x:c r="F15" s="2"/>
-      <x:c r="G15" s="2"/>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="37" t="str">
+        <x:v>Barclays</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>Quantitative Finance Associate Summer Internship Program, 2027 (New York)</x:v>
+      </x:c>
+      <x:c r="C15" s="38" t="n">
+        <x:v>46288</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="str">
+        <x:v>OA received</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="str">
+        <x:v>User-reported OA</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="e">
+        <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Barclays_Quantitative_Analytics_2027.pdf","Open PDF")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Barclays_Quantitative_Analytics_2027.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
+      <x:c r="G15" s="39" t="str">
+        <x:v>Online assessment invitation received.</x:v>
+      </x:c>
       <x:c r="H15" s="2"/>
       <x:c r="I15" s="2"/>
       <x:c r="J15" s="2"/>
       <x:c r="K15" s="2"/>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="2"/>
-      <x:c r="B16" s="2"/>
-      <x:c r="C16" s="2"/>
-      <x:c r="D16" s="2"/>
-      <x:c r="E16" s="2"/>
-      <x:c r="F16" s="2"/>
-      <x:c r="G16" s="2"/>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="40" t="str">
+        <x:v>Balbec Capital LP</x:v>
+      </x:c>
+      <x:c r="B16" s="41" t="str">
+        <x:v>2027 Quantitative Summer Analyst</x:v>
+      </x:c>
+      <x:c r="C16" s="42" t="n">
+        <x:v>46289</x:v>
+      </x:c>
+      <x:c r="D16" s="41" t="str">
+        <x:v>Application received / reviewing</x:v>
+      </x:c>
+      <x:c r="E16" s="41" t="str">
+        <x:v>Direct-portal confirmation email</x:v>
+      </x:c>
+      <x:c r="F16" s="41" t="e">
+        <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Quantitative_Summer_Analyst.pdf","Open PDF")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Quantitative_Summer_Analyst.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
+      <x:c r="G16" s="43" t="str"/>
       <x:c r="H16" s="2"/>
       <x:c r="I16" s="2"/>
       <x:c r="J16" s="2"/>
@@ -3071,10 +3183,12 @@
     <x:mergeCell ref="A2:G2"/>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D6:D14">
-    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Assessment"/>
-    <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="received"/>
-    <x:cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="Submitted"/>
+  <x:conditionalFormatting sqref="D6:D16">
+    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Assessment"/>
+    <x:cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="received"/>
+    <x:cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="Submitted"/>
+    <x:cfRule type="containsText" dxfId="8" priority="4" operator="containsText" text="OA"/>
+    <x:cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="Rejected"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add email-confirmed applications and assessment statuses
</commit_message>
<xml_diff>
--- a/job_application_dashboard_2026-09-24.xlsx
+++ b/job_application_dashboard_2026-09-24.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5669b74fb3f340ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="2" r:id="R7b38526d99f34f35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7903976fe1ef49d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="2" r:id="Ra13a897747bd4559"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -182,7 +182,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="43">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -215,9 +215,6 @@
     <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
@@ -233,11 +230,8 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -291,6 +285,9 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -708,73 +705,74 @@
       <x:c r="K5" s="2"/>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
-      <x:c r="A6" s="13" t="str">
+      <x:c r="A6" s="12" t="str">
         <x:v>Total applications</x:v>
       </x:c>
-      <x:c r="B6" s="14" t="str">
+      <x:c r="B6" s="13" t="str">
         <x:v>Submitted</x:v>
       </x:c>
-      <x:c r="C6" s="14" t="str">
+      <x:c r="C6" s="13" t="str">
         <x:v>Received / reviewing</x:v>
       </x:c>
-      <x:c r="D6" s="14" t="str">
+      <x:c r="D6" s="13" t="str">
+        <x:v>OA received</x:v>
+      </x:c>
+      <x:c r="E6" s="13" t="str">
+        <x:v>OA outstanding</x:v>
+      </x:c>
+      <x:c r="F6" s="13" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="G6" s="13" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="E6" s="14" t="str">
-        <x:v>OA outstanding</x:v>
-      </x:c>
-      <x:c r="F6" s="14" t="str">
-        <x:v>Rejected</x:v>
-      </x:c>
-      <x:c r="G6" s="14" t="str">
+      <x:c r="H6" s="14" t="str">
         <x:v>Latest submission</x:v>
-      </x:c>
-      <x:c r="H6" s="15" t="str">
-        <x:v>Public resume links</x:v>
       </x:c>
       <x:c r="I6" s="2"/>
       <x:c r="J6" s="2"/>
       <x:c r="K6" s="2"/>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
-      <x:c r="A7" s="16" t="n">
+      <x:c r="A7" s="15" t="n">
         <x:f>COUNTA(Applications!A6:A50)</x:f>
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B7" s="17" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="n">
         <x:f>COUNTIFS(Applications!D6:D50,"Submitted")</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C7" s="17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="n">
         <x:f>COUNTIFS(Applications!D6:D50,"Received")+COUNTIFS(Applications!D6:D50,"Received / under review")+COUNTIFS(Applications!D6:D50,"Application received / reviewing")</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D7" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="n">
+        <x:f>COUNTIFS(Applications!D6:D50,"OA received")</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E7" s="16" t="n">
+        <x:f>COUNTIFS(Applications!D6:D50,"OA outstanding")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="n">
+        <x:f>COUNTIFS(Applications!D6:D50,"Rejected")</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="n">
         <x:f>COUNTIFS(Applications!D6:D50,"In Progress")</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E7" s="17" t="n">
-        <x:f>COUNTIFS(Applications!D6:D50,"OA outstanding")</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F7" s="17" t="n">
-        <x:f>COUNTIFS(Applications!D6:D50,"Rejected")</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G7" s="18" t="n">
+      <x:c r="H7" s="17" t="n">
         <x:f>MAX(Applications!C6:C50)</x:f>
         <x:v>46289</x:v>
-      </x:c>
-      <x:c r="H7" s="19" t="str">
-        <x:v>Click Open PDF in the tracker</x:v>
       </x:c>
       <x:c r="I7" s="2"/>
       <x:c r="J7" s="2"/>
       <x:c r="K7" s="2"/>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="20" t="str">
-        <x:v>Evidence combines application logs, candidate portals, confirmation emails, and user-reported outcomes. Balbec appears twice because two confirmed submission channels were recorded.</x:v>
+      <x:c r="A8" s="18" t="str">
+        <x:v>Evidence combines application logs, candidate portals, confirmation emails, and user-reported outcomes. “Not captured” means no role-specific PDF was found locally. Balbec appears twice because two confirmed submission channels were recorded.</x:v>
       </x:c>
       <x:c r="B8" s="2"/>
       <x:c r="C8" s="2"/>
@@ -801,22 +799,22 @@
       <x:c r="K9" s="2"/>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
-      <x:c r="A10" s="34" t="str">
+      <x:c r="A10" s="32" t="str">
         <x:v>Company</x:v>
       </x:c>
-      <x:c r="B10" s="35" t="str">
+      <x:c r="B10" s="33" t="str">
         <x:v>Role</x:v>
       </x:c>
-      <x:c r="C10" s="35" t="str">
+      <x:c r="C10" s="33" t="str">
         <x:v>Submitted</x:v>
       </x:c>
-      <x:c r="D10" s="35" t="str">
+      <x:c r="D10" s="33" t="str">
         <x:v>Current status</x:v>
       </x:c>
-      <x:c r="E10" s="35" t="str">
+      <x:c r="E10" s="33" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="F10" s="36" t="str">
+      <x:c r="F10" s="34" t="str">
         <x:v>Resume</x:v>
       </x:c>
       <x:c r="G10" s="2"/>
@@ -826,27 +824,27 @@
       <x:c r="K10" s="2"/>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
-      <x:c r="A11" s="37" t="str">
+      <x:c r="A11" s="35" t="str">
         <x:f>Applications!A6</x:f>
         <x:v>Arrowstreet Capital</x:v>
       </x:c>
-      <x:c r="B11" s="12" t="str">
+      <x:c r="B11" s="36" t="str">
         <x:f>Applications!B6</x:f>
         <x:v>Quantitative Developer Intern, Summer 2027 (R1506)</x:v>
       </x:c>
-      <x:c r="C11" s="38" t="n">
+      <x:c r="C11" s="37" t="n">
         <x:f>Applications!C6</x:f>
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D11" s="12" t="str">
+      <x:c r="D11" s="36" t="str">
         <x:f>Applications!D6</x:f>
         <x:v>In Progress</x:v>
       </x:c>
-      <x:c r="E11" s="12" t="str">
+      <x:c r="E11" s="36" t="str">
         <x:f>Applications!E6</x:f>
         <x:v>Official candidate home</x:v>
       </x:c>
-      <x:c r="F11" s="39" t="e">
+      <x:c r="F11" s="38" t="e">
         <x:f>Applications!F6</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Arrowstreet_Quant_Developer_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -857,27 +855,27 @@
       <x:c r="K11" s="2"/>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
-      <x:c r="A12" s="37" t="str">
+      <x:c r="A12" s="35" t="str">
         <x:f>Applications!A7</x:f>
         <x:v>Applied Academics LLC</x:v>
       </x:c>
-      <x:c r="B12" s="12" t="str">
+      <x:c r="B12" s="36" t="str">
         <x:f>Applications!B7</x:f>
         <x:v>Quantitative Analyst Intern</x:v>
       </x:c>
-      <x:c r="C12" s="38" t="n">
+      <x:c r="C12" s="37" t="n">
         <x:f>Applications!C7</x:f>
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D12" s="12" t="str">
+      <x:c r="D12" s="36" t="str">
         <x:f>Applications!D7</x:f>
         <x:v>Submitted</x:v>
       </x:c>
-      <x:c r="E12" s="12" t="str">
+      <x:c r="E12" s="36" t="str">
         <x:f>Applications!E7</x:f>
         <x:v>Handshake confirmation</x:v>
       </x:c>
-      <x:c r="F12" s="39" t="e">
+      <x:c r="F12" s="38" t="e">
         <x:f>Applications!F7</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Applied_Academics_Analyst_Intern_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -888,27 +886,27 @@
       <x:c r="K12" s="2"/>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
-      <x:c r="A13" s="37" t="str">
+      <x:c r="A13" s="35" t="str">
         <x:f>Applications!A8</x:f>
-        <x:v>IMC</x:v>
-      </x:c>
-      <x:c r="B13" s="12" t="str">
+        <x:v>IMC Trading</x:v>
+      </x:c>
+      <x:c r="B13" s="36" t="str">
         <x:f>Applications!B8</x:f>
-        <x:v>Quantitative Trader Intern, Summer 2027 (Chicago)</x:v>
-      </x:c>
-      <x:c r="C13" s="38" t="n">
+        <x:v>Quantitative Trader Intern, Summer 2027</x:v>
+      </x:c>
+      <x:c r="C13" s="37" t="n">
         <x:f>Applications!C8</x:f>
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D13" s="12" t="str">
+      <x:c r="D13" s="36" t="str">
         <x:f>Applications!D8</x:f>
-        <x:v>Submitted</x:v>
-      </x:c>
-      <x:c r="E13" s="12" t="str">
+        <x:v>OA received</x:v>
+      </x:c>
+      <x:c r="E13" s="36" t="str">
         <x:f>Applications!E8</x:f>
-        <x:v>Official confirmation page</x:v>
-      </x:c>
-      <x:c r="F13" s="39" t="e">
+        <x:v>IMC / SHL assessment invitations</x:v>
+      </x:c>
+      <x:c r="F13" s="38" t="e">
         <x:f>Applications!F8</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.IMC_Trader_Intern_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -919,27 +917,27 @@
       <x:c r="K13" s="2"/>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
-      <x:c r="A14" s="37" t="str">
+      <x:c r="A14" s="35" t="str">
         <x:f>Applications!A9</x:f>
         <x:v>Balbec Capital LP</x:v>
       </x:c>
-      <x:c r="B14" s="12" t="str">
+      <x:c r="B14" s="36" t="str">
         <x:f>Applications!B9</x:f>
         <x:v>2027 Quantitative Summer Analyst</x:v>
       </x:c>
-      <x:c r="C14" s="38" t="n">
+      <x:c r="C14" s="37" t="n">
         <x:f>Applications!C9</x:f>
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D14" s="12" t="str">
+      <x:c r="D14" s="36" t="str">
         <x:f>Applications!D9</x:f>
         <x:v>Submitted</x:v>
       </x:c>
-      <x:c r="E14" s="12" t="str">
+      <x:c r="E14" s="36" t="str">
         <x:f>Applications!E9</x:f>
         <x:v>Handshake confirmation</x:v>
       </x:c>
-      <x:c r="F14" s="39" t="e">
+      <x:c r="F14" s="38" t="e">
         <x:f>Applications!F9</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Summer_Analyst_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -950,27 +948,27 @@
       <x:c r="K14" s="2"/>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
-      <x:c r="A15" s="37" t="str">
+      <x:c r="A15" s="35" t="str">
         <x:f>Applications!A10</x:f>
         <x:v>Walleye Capital</x:v>
       </x:c>
-      <x:c r="B15" s="12" t="str">
+      <x:c r="B15" s="36" t="str">
         <x:f>Applications!B10</x:f>
         <x:v>Quantitative Developer Intern, Summer 2027</x:v>
       </x:c>
-      <x:c r="C15" s="38" t="n">
+      <x:c r="C15" s="37" t="n">
         <x:f>Applications!C10</x:f>
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D15" s="12" t="str">
+      <x:c r="D15" s="36" t="str">
         <x:f>Applications!D10</x:f>
         <x:v>Received / under review</x:v>
       </x:c>
-      <x:c r="E15" s="12" t="str">
+      <x:c r="E15" s="36" t="str">
         <x:f>Applications!E10</x:f>
         <x:v>Official confirmation page</x:v>
       </x:c>
-      <x:c r="F15" s="39" t="e">
+      <x:c r="F15" s="38" t="e">
         <x:f>Applications!F10</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Walleye_Quantic_Developer_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -981,27 +979,27 @@
       <x:c r="K15" s="2"/>
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
-      <x:c r="A16" s="37" t="str">
+      <x:c r="A16" s="35" t="str">
         <x:f>Applications!A11</x:f>
         <x:v>Seven Research</x:v>
       </x:c>
-      <x:c r="B16" s="12" t="str">
+      <x:c r="B16" s="36" t="str">
         <x:f>Applications!B11</x:f>
         <x:v>Quantitative Researcher Intern</x:v>
       </x:c>
-      <x:c r="C16" s="38" t="n">
+      <x:c r="C16" s="37" t="n">
         <x:f>Applications!C11</x:f>
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D16" s="12" t="str">
+      <x:c r="D16" s="36" t="str">
         <x:f>Applications!D11</x:f>
         <x:v>Received</x:v>
       </x:c>
-      <x:c r="E16" s="12" t="str">
+      <x:c r="E16" s="36" t="str">
         <x:f>Applications!E11</x:f>
         <x:v>Official confirmation page</x:v>
       </x:c>
-      <x:c r="F16" s="39" t="e">
+      <x:c r="F16" s="38" t="e">
         <x:f>Applications!F11</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Seven_Research_Quant_Researcher_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -1012,27 +1010,27 @@
       <x:c r="K16" s="2"/>
     </x:row>
     <x:row r="17" ht="20" customHeight="1">
-      <x:c r="A17" s="37" t="str">
+      <x:c r="A17" s="35" t="str">
         <x:f>Applications!A12</x:f>
         <x:v>Bank of America</x:v>
       </x:c>
-      <x:c r="B17" s="12" t="str">
+      <x:c r="B17" s="36" t="str">
         <x:f>Applications!B12</x:f>
         <x:v>Global Quantitative Research Summer Associate Program, 2027</x:v>
       </x:c>
-      <x:c r="C17" s="38" t="n">
+      <x:c r="C17" s="37" t="n">
         <x:f>Applications!C12</x:f>
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D17" s="12" t="str">
+      <x:c r="D17" s="36" t="str">
         <x:f>Applications!D12</x:f>
         <x:v>OA outstanding</x:v>
       </x:c>
-      <x:c r="E17" s="12" t="str">
+      <x:c r="E17" s="36" t="str">
         <x:f>Applications!E12</x:f>
         <x:v>Application Center</x:v>
       </x:c>
-      <x:c r="F17" s="39" t="e">
+      <x:c r="F17" s="38" t="e">
         <x:f>Applications!F12</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.BofA_Global_Quant_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -1043,27 +1041,27 @@
       <x:c r="K17" s="2"/>
     </x:row>
     <x:row r="18" ht="20" customHeight="1">
-      <x:c r="A18" s="37" t="str">
+      <x:c r="A18" s="35" t="str">
         <x:f>Applications!A13</x:f>
         <x:v>Fidelity Investments</x:v>
       </x:c>
-      <x:c r="B18" s="12" t="str">
+      <x:c r="B18" s="36" t="str">
         <x:f>Applications!B13</x:f>
         <x:v>Quantitative Research Intern, Multi-Asset Systematic Research Team</x:v>
       </x:c>
-      <x:c r="C18" s="38" t="n">
+      <x:c r="C18" s="37" t="n">
         <x:f>Applications!C13</x:f>
         <x:v>46287</x:v>
       </x:c>
-      <x:c r="D18" s="12" t="str">
+      <x:c r="D18" s="36" t="str">
         <x:f>Applications!D13</x:f>
         <x:v>Rejected</x:v>
       </x:c>
-      <x:c r="E18" s="12" t="str">
+      <x:c r="E18" s="36" t="str">
         <x:f>Applications!E13</x:f>
         <x:v>User-reported outcome</x:v>
       </x:c>
-      <x:c r="F18" s="39" t="e">
+      <x:c r="F18" s="38" t="e">
         <x:f>Applications!F13</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Multi_Asset_Systematic_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -1074,27 +1072,27 @@
       <x:c r="K18" s="2"/>
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
-      <x:c r="A19" s="37" t="str">
+      <x:c r="A19" s="35" t="str">
         <x:f>Applications!A14</x:f>
         <x:v>Fidelity Investments</x:v>
       </x:c>
-      <x:c r="B19" s="12" t="str">
+      <x:c r="B19" s="36" t="str">
         <x:f>Applications!B14</x:f>
         <x:v>Quantitative Research Intern, Fixed Income Team</x:v>
       </x:c>
-      <x:c r="C19" s="38" t="n">
+      <x:c r="C19" s="37" t="n">
         <x:f>Applications!C14</x:f>
         <x:v>46287</x:v>
       </x:c>
-      <x:c r="D19" s="12" t="str">
+      <x:c r="D19" s="36" t="str">
         <x:f>Applications!D14</x:f>
         <x:v>Rejected</x:v>
       </x:c>
-      <x:c r="E19" s="12" t="str">
+      <x:c r="E19" s="36" t="str">
         <x:f>Applications!E14</x:f>
         <x:v>User-reported outcome</x:v>
       </x:c>
-      <x:c r="F19" s="39" t="e">
+      <x:c r="F19" s="38" t="e">
         <x:f>Applications!F14</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Fixed_Income_Quantitative_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -1105,27 +1103,27 @@
       <x:c r="K19" s="2"/>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
-      <x:c r="A20" s="37" t="str">
+      <x:c r="A20" s="35" t="str">
         <x:f>Applications!A15</x:f>
         <x:v>Barclays</x:v>
       </x:c>
-      <x:c r="B20" s="12" t="str">
+      <x:c r="B20" s="36" t="str">
         <x:f>Applications!B15</x:f>
         <x:v>Quantitative Finance Associate Summer Internship Program, 2027 (New York)</x:v>
       </x:c>
-      <x:c r="C20" s="38" t="n">
+      <x:c r="C20" s="37" t="n">
         <x:f>Applications!C15</x:f>
         <x:v>46288</x:v>
       </x:c>
-      <x:c r="D20" s="12" t="str">
+      <x:c r="D20" s="36" t="str">
         <x:f>Applications!D15</x:f>
         <x:v>OA received</x:v>
       </x:c>
-      <x:c r="E20" s="12" t="str">
+      <x:c r="E20" s="36" t="str">
         <x:f>Applications!E15</x:f>
         <x:v>User-reported OA</x:v>
       </x:c>
-      <x:c r="F20" s="39" t="e">
+      <x:c r="F20" s="38" t="e">
         <x:f>Applications!F15</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Barclays_Quantitative_Analytics_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -1136,27 +1134,27 @@
       <x:c r="K20" s="2"/>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
-      <x:c r="A21" s="40" t="str">
+      <x:c r="A21" s="35" t="str">
         <x:f>Applications!A16</x:f>
         <x:v>Balbec Capital LP</x:v>
       </x:c>
-      <x:c r="B21" s="41" t="str">
+      <x:c r="B21" s="36" t="str">
         <x:f>Applications!B16</x:f>
         <x:v>2027 Quantitative Summer Analyst</x:v>
       </x:c>
-      <x:c r="C21" s="42" t="n">
+      <x:c r="C21" s="37" t="n">
         <x:f>Applications!C16</x:f>
         <x:v>46289</x:v>
       </x:c>
-      <x:c r="D21" s="41" t="str">
+      <x:c r="D21" s="36" t="str">
         <x:f>Applications!D16</x:f>
         <x:v>Application received / reviewing</x:v>
       </x:c>
-      <x:c r="E21" s="41" t="str">
+      <x:c r="E21" s="36" t="str">
         <x:f>Applications!E16</x:f>
         <x:v>Direct-portal confirmation email</x:v>
       </x:c>
-      <x:c r="F21" s="43" t="e">
+      <x:c r="F21" s="38" t="e">
         <x:f>Applications!F16</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Quantitative_Summer_Analyst.pdf, friendlyName=Open PDF</x:v>
       </x:c>
@@ -1167,12 +1165,30 @@
       <x:c r="K21" s="2"/>
     </x:row>
     <x:row r="22" ht="20" customHeight="1">
-      <x:c r="A22" s="2"/>
-      <x:c r="B22" s="2"/>
-      <x:c r="C22" s="2"/>
-      <x:c r="D22" s="2"/>
-      <x:c r="E22" s="2"/>
-      <x:c r="F22" s="2"/>
+      <x:c r="A22" s="35" t="str">
+        <x:f>Applications!A17</x:f>
+        <x:v>Millennium Management</x:v>
+      </x:c>
+      <x:c r="B22" s="36" t="str">
+        <x:f>Applications!B17</x:f>
+        <x:v>2027 Quantitative Researcher Intern, New York</x:v>
+      </x:c>
+      <x:c r="C22" s="37" t="n">
+        <x:f>Applications!C17</x:f>
+        <x:v>46263</x:v>
+      </x:c>
+      <x:c r="D22" s="36" t="str">
+        <x:f>Applications!D17</x:f>
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E22" s="36" t="str">
+        <x:f>Applications!E17</x:f>
+        <x:v>Workday receipt and candidacy update</x:v>
+      </x:c>
+      <x:c r="F22" s="38" t="str">
+        <x:f>Applications!F17</x:f>
+        <x:v>Not captured</x:v>
+      </x:c>
       <x:c r="G22" s="2"/>
       <x:c r="H22" s="2"/>
       <x:c r="I22" s="2"/>
@@ -1180,86 +1196,192 @@
       <x:c r="K22" s="2"/>
     </x:row>
     <x:row r="23" ht="20" customHeight="1">
-      <x:c r="A23" s="2"/>
-      <x:c r="B23" s="2"/>
-      <x:c r="C23" s="2"/>
-      <x:c r="D23" s="2"/>
-      <x:c r="E23" s="2"/>
-      <x:c r="F23" s="2"/>
+      <x:c r="A23" s="35" t="str">
+        <x:f>Applications!A18</x:f>
+        <x:v>Millennium Management</x:v>
+      </x:c>
+      <x:c r="B23" s="36" t="str">
+        <x:f>Applications!B18</x:f>
+        <x:v>2027 Quantitative Developer Intern, New York</x:v>
+      </x:c>
+      <x:c r="C23" s="37" t="n">
+        <x:f>Applications!C18</x:f>
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="D23" s="36" t="str">
+        <x:f>Applications!D18</x:f>
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E23" s="36" t="str">
+        <x:f>Applications!E18</x:f>
+        <x:v>Workday receipt and candidacy update</x:v>
+      </x:c>
+      <x:c r="F23" s="38" t="str">
+        <x:f>Applications!F18</x:f>
+        <x:v>Not captured</x:v>
+      </x:c>
       <x:c r="G23" s="2"/>
       <x:c r="H23" s="2"/>
       <x:c r="I23" s="2"/>
       <x:c r="J23" s="2"/>
       <x:c r="K23" s="2"/>
     </x:row>
-    <x:row r="24" ht="26" customHeight="1">
-      <x:c r="A24"/>
-      <x:c r="B24" s="2"/>
-      <x:c r="C24" s="2"/>
-      <x:c r="D24" s="2"/>
-      <x:c r="E24" s="2"/>
-      <x:c r="F24" s="2"/>
+    <x:row r="24" ht="20" customHeight="1">
+      <x:c r="A24" s="35" t="str">
+        <x:f>Applications!A19</x:f>
+        <x:v>D. E. Shaw</x:v>
+      </x:c>
+      <x:c r="B24" s="36" t="str">
+        <x:f>Applications!B19</x:f>
+        <x:v>Quantitative Analyst Intern, New York, Summer 2027</x:v>
+      </x:c>
+      <x:c r="C24" s="37" t="n">
+        <x:f>Applications!C19</x:f>
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="D24" s="36" t="str">
+        <x:f>Applications!D19</x:f>
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E24" s="36" t="str">
+        <x:f>Applications!E19</x:f>
+        <x:v>Application receipt and employer update</x:v>
+      </x:c>
+      <x:c r="F24" s="38" t="e">
+        <x:f>Applications!F19</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.DE_Shaw_Quantitative_Analyst_Intern.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
       <x:c r="G24" s="2"/>
       <x:c r="H24" s="2"/>
       <x:c r="I24" s="2"/>
       <x:c r="J24" s="2"/>
       <x:c r="K24" s="2"/>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="2"/>
-      <x:c r="B25" s="2"/>
-      <x:c r="C25" s="2"/>
-      <x:c r="D25" s="2"/>
-      <x:c r="E25" s="2"/>
-      <x:c r="F25" s="2"/>
+    <x:row r="25" ht="20" customHeight="1">
+      <x:c r="A25" s="35" t="str">
+        <x:f>Applications!A20</x:f>
+        <x:v>Jane Street</x:v>
+      </x:c>
+      <x:c r="B25" s="36" t="str">
+        <x:f>Applications!B20</x:f>
+        <x:v>Role not specified in employer email</x:v>
+      </x:c>
+      <x:c r="C25" s="37" t="n">
+        <x:f>Applications!C20</x:f>
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="D25" s="36" t="str">
+        <x:f>Applications!D20</x:f>
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E25" s="36" t="str">
+        <x:f>Applications!E20</x:f>
+        <x:v>Receipt and employer update</x:v>
+      </x:c>
+      <x:c r="F25" s="38" t="e">
+        <x:f>Applications!F20</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Jane_Street_Quantitative_Researcher_Intern.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
       <x:c r="G25" s="2"/>
       <x:c r="H25" s="2"/>
       <x:c r="I25" s="2"/>
       <x:c r="J25" s="2"/>
       <x:c r="K25" s="2"/>
     </x:row>
-    <x:row r="26" ht="26" customHeight="1">
-      <x:c r="A26" s="20" t="str">
-        <x:v>Definitions: “Submitted” is a completed application. “Received / reviewing” is an employer acknowledgment. “OA outstanding” means an online assessment remains to be completed. “OA received” means the assessment invitation has been received.</x:v>
-      </x:c>
-      <x:c r="B26" s="2"/>
-      <x:c r="C26" s="2"/>
-      <x:c r="D26" s="2"/>
-      <x:c r="E26" s="2"/>
-      <x:c r="F26" s="2"/>
+    <x:row r="26" ht="20" customHeight="1">
+      <x:c r="A26" s="35" t="str">
+        <x:f>Applications!A21</x:f>
+        <x:v>Ridgeline</x:v>
+      </x:c>
+      <x:c r="B26" s="36" t="str">
+        <x:f>Applications!B21</x:f>
+        <x:v>Software Engineer Intern, Summer 2027 (Cornell)</x:v>
+      </x:c>
+      <x:c r="C26" s="37" t="n">
+        <x:f>Applications!C21</x:f>
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="D26" s="36" t="str">
+        <x:f>Applications!D21</x:f>
+        <x:v>Received / under review</x:v>
+      </x:c>
+      <x:c r="E26" s="36" t="str">
+        <x:f>Applications!E21</x:f>
+        <x:v>Greenhouse confirmation email</x:v>
+      </x:c>
+      <x:c r="F26" s="38" t="str">
+        <x:f>Applications!F21</x:f>
+        <x:v>Not captured</x:v>
+      </x:c>
       <x:c r="G26" s="2"/>
       <x:c r="H26" s="2"/>
       <x:c r="I26" s="2"/>
       <x:c r="J26" s="2"/>
       <x:c r="K26" s="2"/>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="2"/>
-      <x:c r="B27" s="2"/>
-      <x:c r="C27" s="2"/>
-      <x:c r="D27" s="2"/>
-      <x:c r="E27" s="2"/>
-      <x:c r="F27" s="2"/>
+    <x:row r="27" ht="20" customHeight="1">
+      <x:c r="A27" s="35" t="str">
+        <x:f>Applications!A22</x:f>
+        <x:v>Susquehanna</x:v>
+      </x:c>
+      <x:c r="B27" s="36" t="str">
+        <x:f>Applications!B22</x:f>
+        <x:v>Quantitative Research position</x:v>
+      </x:c>
+      <x:c r="C27" s="37" t="n">
+        <x:f>Applications!C22</x:f>
+        <x:v>46274</x:v>
+      </x:c>
+      <x:c r="D27" s="36" t="str">
+        <x:f>Applications!D22</x:f>
+        <x:v>OA received</x:v>
+      </x:c>
+      <x:c r="E27" s="36" t="str">
+        <x:f>Applications!E22</x:f>
+        <x:v>Recruiting and Mettl assessment invitations</x:v>
+      </x:c>
+      <x:c r="F27" s="38" t="e">
+        <x:f>Applications!F22</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Susquehanna_Quantitative_Research_Intern.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
       <x:c r="G27" s="2"/>
       <x:c r="H27" s="2"/>
       <x:c r="I27" s="2"/>
       <x:c r="J27" s="2"/>
       <x:c r="K27" s="2"/>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="2"/>
-      <x:c r="B28" s="2"/>
-      <x:c r="C28" s="2"/>
-      <x:c r="D28" s="2"/>
-      <x:c r="E28" s="2"/>
-      <x:c r="F28" s="2"/>
+    <x:row r="28" ht="20" customHeight="1">
+      <x:c r="A28" s="39" t="str">
+        <x:f>Applications!A23</x:f>
+        <x:v>Susquehanna</x:v>
+      </x:c>
+      <x:c r="B28" s="40" t="str">
+        <x:f>Applications!B23</x:f>
+        <x:v>Quantitative Systematic Trading position</x:v>
+      </x:c>
+      <x:c r="C28" s="41" t="n">
+        <x:f>Applications!C23</x:f>
+        <x:v>46274</x:v>
+      </x:c>
+      <x:c r="D28" s="40" t="str">
+        <x:f>Applications!D23</x:f>
+        <x:v>OA received</x:v>
+      </x:c>
+      <x:c r="E28" s="40" t="str">
+        <x:f>Applications!E23</x:f>
+        <x:v>Recruiting and Mettl assessment invitations</x:v>
+      </x:c>
+      <x:c r="F28" s="42" t="str">
+        <x:f>Applications!F23</x:f>
+        <x:v>Not captured</x:v>
+      </x:c>
       <x:c r="G28" s="2"/>
       <x:c r="H28" s="2"/>
       <x:c r="I28" s="2"/>
       <x:c r="J28" s="2"/>
       <x:c r="K28" s="2"/>
     </x:row>
-    <x:row r="29">
+    <x:row r="29" ht="20" customHeight="1">
       <x:c r="A29" s="2"/>
       <x:c r="B29" s="2"/>
       <x:c r="C29" s="2"/>
@@ -1272,7 +1394,7 @@
       <x:c r="J29" s="2"/>
       <x:c r="K29" s="2"/>
     </x:row>
-    <x:row r="30">
+    <x:row r="30" ht="20" customHeight="1">
       <x:c r="A30" s="2"/>
       <x:c r="B30" s="2"/>
       <x:c r="C30" s="2"/>
@@ -1285,7 +1407,7 @@
       <x:c r="J30" s="2"/>
       <x:c r="K30" s="2"/>
     </x:row>
-    <x:row r="31">
+    <x:row r="31" ht="20" customHeight="1">
       <x:c r="A31" s="2"/>
       <x:c r="B31" s="2"/>
       <x:c r="C31" s="2"/>
@@ -1298,7 +1420,7 @@
       <x:c r="J31" s="2"/>
       <x:c r="K31" s="2"/>
     </x:row>
-    <x:row r="32">
+    <x:row r="32" ht="20" customHeight="1">
       <x:c r="A32" s="2"/>
       <x:c r="B32" s="2"/>
       <x:c r="C32" s="2"/>
@@ -1311,8 +1433,10 @@
       <x:c r="J32" s="2"/>
       <x:c r="K32" s="2"/>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="2"/>
+    <x:row r="33" ht="26" customHeight="1">
+      <x:c r="A33" s="18" t="str">
+        <x:v>Definitions: “Submitted” is a completed application. “Received / reviewing” is an employer acknowledgment. “OA outstanding” means an online assessment remains to be completed. “OA received” means the assessment invitation has been received.</x:v>
+      </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
       <x:c r="D33" s="2"/>
@@ -1940,9 +2064,9 @@
     <x:mergeCell ref="A2:H2"/>
     <x:mergeCell ref="A3:H3"/>
     <x:mergeCell ref="A8:H8"/>
-    <x:mergeCell ref="A26:H26"/>
+    <x:mergeCell ref="A33:H33"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D11:D21">
+  <x:conditionalFormatting sqref="D11:D28">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Assessment"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="received"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Submitted"/>
@@ -2026,25 +2150,25 @@
       <x:c r="K4" s="2"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="34" t="str">
+      <x:c r="A5" s="32" t="str">
         <x:v>Company</x:v>
       </x:c>
-      <x:c r="B5" s="35" t="str">
+      <x:c r="B5" s="33" t="str">
         <x:v>Role</x:v>
       </x:c>
-      <x:c r="C5" s="35" t="str">
+      <x:c r="C5" s="33" t="str">
         <x:v>Application date</x:v>
       </x:c>
-      <x:c r="D5" s="35" t="str">
+      <x:c r="D5" s="33" t="str">
         <x:v>Current status</x:v>
       </x:c>
-      <x:c r="E5" s="35" t="str">
+      <x:c r="E5" s="33" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="F5" s="35" t="str">
+      <x:c r="F5" s="33" t="str">
         <x:v>Resume PDF</x:v>
       </x:c>
-      <x:c r="G5" s="36" t="str">
+      <x:c r="G5" s="34" t="str">
         <x:v>Notes</x:v>
       </x:c>
       <x:c r="H5" s="2"/>
@@ -2053,182 +2177,184 @@
       <x:c r="K5" s="2"/>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="37" t="str">
+      <x:c r="A6" s="35" t="str">
         <x:v>Arrowstreet Capital</x:v>
       </x:c>
-      <x:c r="B6" s="12" t="str">
+      <x:c r="B6" s="36" t="str">
         <x:v>Quantitative Developer Intern, Summer 2027 (R1506)</x:v>
       </x:c>
-      <x:c r="C6" s="38" t="n">
+      <x:c r="C6" s="37" t="n">
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D6" s="12" t="str">
+      <x:c r="D6" s="36" t="str">
         <x:v>In Progress</x:v>
       </x:c>
-      <x:c r="E6" s="12" t="str">
+      <x:c r="E6" s="36" t="str">
         <x:v>Official candidate home</x:v>
       </x:c>
-      <x:c r="F6" s="12" t="e">
+      <x:c r="F6" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Arrowstreet_Quant_Developer_Intern.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Arrowstreet_Quant_Developer_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G6" s="39" t="str"/>
+      <x:c r="G6" s="38" t="str"/>
       <x:c r="H6" s="2"/>
       <x:c r="I6" s="2"/>
       <x:c r="J6" s="2"/>
       <x:c r="K6" s="2"/>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="37" t="str">
+      <x:c r="A7" s="35" t="str">
         <x:v>Applied Academics LLC</x:v>
       </x:c>
-      <x:c r="B7" s="12" t="str">
+      <x:c r="B7" s="36" t="str">
         <x:v>Quantitative Analyst Intern</x:v>
       </x:c>
-      <x:c r="C7" s="38" t="n">
+      <x:c r="C7" s="37" t="n">
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D7" s="12" t="str">
+      <x:c r="D7" s="36" t="str">
         <x:v>Submitted</x:v>
       </x:c>
-      <x:c r="E7" s="12" t="str">
+      <x:c r="E7" s="36" t="str">
         <x:v>Handshake confirmation</x:v>
       </x:c>
-      <x:c r="F7" s="12" t="e">
+      <x:c r="F7" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Applied_Academics_Analyst_Intern_JD.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Applied_Academics_Analyst_Intern_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G7" s="39" t="str"/>
+      <x:c r="G7" s="38" t="str"/>
       <x:c r="H7" s="2"/>
       <x:c r="I7" s="2"/>
       <x:c r="J7" s="2"/>
       <x:c r="K7" s="2"/>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="37" t="str">
-        <x:v>IMC</x:v>
-      </x:c>
-      <x:c r="B8" s="12" t="str">
-        <x:v>Quantitative Trader Intern, Summer 2027 (Chicago)</x:v>
-      </x:c>
-      <x:c r="C8" s="38" t="n">
+      <x:c r="A8" s="35" t="str">
+        <x:v>IMC Trading</x:v>
+      </x:c>
+      <x:c r="B8" s="36" t="str">
+        <x:v>Quantitative Trader Intern, Summer 2027</x:v>
+      </x:c>
+      <x:c r="C8" s="37" t="n">
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D8" s="12" t="str">
-        <x:v>Submitted</x:v>
-      </x:c>
-      <x:c r="E8" s="12" t="str">
-        <x:v>Official confirmation page</x:v>
-      </x:c>
-      <x:c r="F8" s="12" t="e">
+      <x:c r="D8" s="36" t="str">
+        <x:v>OA received</x:v>
+      </x:c>
+      <x:c r="E8" s="36" t="str">
+        <x:v>IMC / SHL assessment invitations</x:v>
+      </x:c>
+      <x:c r="F8" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.IMC_Trader_Intern_JD.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.IMC_Trader_Intern_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G8" s="39" t="str"/>
+      <x:c r="G8" s="38" t="str">
+        <x:v>SHL assessment invitation received.</x:v>
+      </x:c>
       <x:c r="H8" s="2"/>
       <x:c r="I8" s="2"/>
       <x:c r="J8" s="2"/>
       <x:c r="K8" s="2"/>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="37" t="str">
+      <x:c r="A9" s="35" t="str">
         <x:v>Balbec Capital LP</x:v>
       </x:c>
-      <x:c r="B9" s="12" t="str">
+      <x:c r="B9" s="36" t="str">
         <x:v>2027 Quantitative Summer Analyst</x:v>
       </x:c>
-      <x:c r="C9" s="38" t="n">
+      <x:c r="C9" s="37" t="n">
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D9" s="12" t="str">
+      <x:c r="D9" s="36" t="str">
         <x:v>Submitted</x:v>
       </x:c>
-      <x:c r="E9" s="12" t="str">
+      <x:c r="E9" s="36" t="str">
         <x:v>Handshake confirmation</x:v>
       </x:c>
-      <x:c r="F9" s="12" t="e">
+      <x:c r="F9" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Summer_Analyst_JD.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Summer_Analyst_JD.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G9" s="39" t="str"/>
+      <x:c r="G9" s="38" t="str"/>
       <x:c r="H9" s="2"/>
       <x:c r="I9" s="2"/>
       <x:c r="J9" s="2"/>
       <x:c r="K9" s="2"/>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="37" t="str">
+      <x:c r="A10" s="35" t="str">
         <x:v>Walleye Capital</x:v>
       </x:c>
-      <x:c r="B10" s="12" t="str">
+      <x:c r="B10" s="36" t="str">
         <x:v>Quantitative Developer Intern, Summer 2027</x:v>
       </x:c>
-      <x:c r="C10" s="38" t="n">
+      <x:c r="C10" s="37" t="n">
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D10" s="12" t="str">
+      <x:c r="D10" s="36" t="str">
         <x:v>Received / under review</x:v>
       </x:c>
-      <x:c r="E10" s="12" t="str">
+      <x:c r="E10" s="36" t="str">
         <x:v>Official confirmation page</x:v>
       </x:c>
-      <x:c r="F10" s="12" t="e">
+      <x:c r="F10" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Walleye_Quantic_Developer_Intern.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Walleye_Quantic_Developer_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G10" s="39" t="str"/>
+      <x:c r="G10" s="38" t="str"/>
       <x:c r="H10" s="2"/>
       <x:c r="I10" s="2"/>
       <x:c r="J10" s="2"/>
       <x:c r="K10" s="2"/>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="37" t="str">
+      <x:c r="A11" s="35" t="str">
         <x:v>Seven Research</x:v>
       </x:c>
-      <x:c r="B11" s="12" t="str">
+      <x:c r="B11" s="36" t="str">
         <x:v>Quantitative Researcher Intern</x:v>
       </x:c>
-      <x:c r="C11" s="38" t="n">
+      <x:c r="C11" s="37" t="n">
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D11" s="12" t="str">
+      <x:c r="D11" s="36" t="str">
         <x:v>Received</x:v>
       </x:c>
-      <x:c r="E11" s="12" t="str">
+      <x:c r="E11" s="36" t="str">
         <x:v>Official confirmation page</x:v>
       </x:c>
-      <x:c r="F11" s="12" t="e">
+      <x:c r="F11" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Seven_Research_Quant_Researcher_Intern.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Seven_Research_Quant_Researcher_Intern.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G11" s="39" t="str"/>
+      <x:c r="G11" s="38" t="str"/>
       <x:c r="H11" s="2"/>
       <x:c r="I11" s="2"/>
       <x:c r="J11" s="2"/>
       <x:c r="K11" s="2"/>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
-      <x:c r="A12" s="37" t="str">
+      <x:c r="A12" s="35" t="str">
         <x:v>Bank of America</x:v>
       </x:c>
-      <x:c r="B12" s="12" t="str">
+      <x:c r="B12" s="36" t="str">
         <x:v>Global Quantitative Research Summer Associate Program, 2027</x:v>
       </x:c>
-      <x:c r="C12" s="38" t="n">
+      <x:c r="C12" s="37" t="n">
         <x:v>46279</x:v>
       </x:c>
-      <x:c r="D12" s="12" t="str">
+      <x:c r="D12" s="36" t="str">
         <x:v>OA outstanding</x:v>
       </x:c>
-      <x:c r="E12" s="12" t="str">
+      <x:c r="E12" s="36" t="str">
         <x:v>Application Center</x:v>
       </x:c>
-      <x:c r="F12" s="12" t="e">
+      <x:c r="F12" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.BofA_Global_Quant_Research_2027.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.BofA_Global_Quant_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G12" s="39" t="str">
+      <x:c r="G12" s="38" t="str">
         <x:v>Application submitted; the employer's online assessment is still required.</x:v>
       </x:c>
       <x:c r="H12" s="2"/>
@@ -2237,26 +2363,26 @@
       <x:c r="K12" s="2"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="37" t="str">
+      <x:c r="A13" s="35" t="str">
         <x:v>Fidelity Investments</x:v>
       </x:c>
-      <x:c r="B13" s="12" t="str">
+      <x:c r="B13" s="36" t="str">
         <x:v>Quantitative Research Intern, Multi-Asset Systematic Research Team</x:v>
       </x:c>
-      <x:c r="C13" s="38" t="n">
+      <x:c r="C13" s="37" t="n">
         <x:v>46287</x:v>
       </x:c>
-      <x:c r="D13" s="12" t="str">
+      <x:c r="D13" s="36" t="str">
         <x:v>Rejected</x:v>
       </x:c>
-      <x:c r="E13" s="12" t="str">
+      <x:c r="E13" s="36" t="str">
         <x:v>User-reported outcome</x:v>
       </x:c>
-      <x:c r="F13" s="12" t="e">
+      <x:c r="F13" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Multi_Asset_Systematic_Research_2027.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Multi_Asset_Systematic_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G13" s="39" t="str">
+      <x:c r="G13" s="38" t="str">
         <x:v>Application outcome reported as rejected.</x:v>
       </x:c>
       <x:c r="H13" s="2"/>
@@ -2265,26 +2391,26 @@
       <x:c r="K13" s="2"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="37" t="str">
+      <x:c r="A14" s="35" t="str">
         <x:v>Fidelity Investments</x:v>
       </x:c>
-      <x:c r="B14" s="12" t="str">
+      <x:c r="B14" s="36" t="str">
         <x:v>Quantitative Research Intern, Fixed Income Team</x:v>
       </x:c>
-      <x:c r="C14" s="38" t="n">
+      <x:c r="C14" s="37" t="n">
         <x:v>46287</x:v>
       </x:c>
-      <x:c r="D14" s="12" t="str">
+      <x:c r="D14" s="36" t="str">
         <x:v>Rejected</x:v>
       </x:c>
-      <x:c r="E14" s="12" t="str">
+      <x:c r="E14" s="36" t="str">
         <x:v>User-reported outcome</x:v>
       </x:c>
-      <x:c r="F14" s="12" t="e">
+      <x:c r="F14" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Fixed_Income_Quantitative_Research_2027.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Fidelity_Fixed_Income_Quantitative_Research_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G14" s="39" t="str">
+      <x:c r="G14" s="38" t="str">
         <x:v>Application outcome reported as rejected.</x:v>
       </x:c>
       <x:c r="H14" s="2"/>
@@ -2293,26 +2419,26 @@
       <x:c r="K14" s="2"/>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="37" t="str">
+      <x:c r="A15" s="35" t="str">
         <x:v>Barclays</x:v>
       </x:c>
-      <x:c r="B15" s="12" t="str">
+      <x:c r="B15" s="36" t="str">
         <x:v>Quantitative Finance Associate Summer Internship Program, 2027 (New York)</x:v>
       </x:c>
-      <x:c r="C15" s="38" t="n">
+      <x:c r="C15" s="37" t="n">
         <x:v>46288</x:v>
       </x:c>
-      <x:c r="D15" s="12" t="str">
+      <x:c r="D15" s="36" t="str">
         <x:v>OA received</x:v>
       </x:c>
-      <x:c r="E15" s="12" t="str">
+      <x:c r="E15" s="36" t="str">
         <x:v>User-reported OA</x:v>
       </x:c>
-      <x:c r="F15" s="12" t="e">
+      <x:c r="F15" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Barclays_Quantitative_Analytics_2027.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Barclays_Quantitative_Analytics_2027.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G15" s="39" t="str">
+      <x:c r="G15" s="38" t="str">
         <x:v>Online assessment invitation received.</x:v>
       </x:c>
       <x:c r="H15" s="2"/>
@@ -2321,117 +2447,216 @@
       <x:c r="K15" s="2"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="40" t="str">
+      <x:c r="A16" s="35" t="str">
         <x:v>Balbec Capital LP</x:v>
       </x:c>
-      <x:c r="B16" s="41" t="str">
+      <x:c r="B16" s="36" t="str">
         <x:v>2027 Quantitative Summer Analyst</x:v>
       </x:c>
-      <x:c r="C16" s="42" t="n">
+      <x:c r="C16" s="37" t="n">
         <x:v>46289</x:v>
       </x:c>
-      <x:c r="D16" s="41" t="str">
+      <x:c r="D16" s="36" t="str">
         <x:v>Application received / reviewing</x:v>
       </x:c>
-      <x:c r="E16" s="41" t="str">
+      <x:c r="E16" s="36" t="str">
         <x:v>Direct-portal confirmation email</x:v>
       </x:c>
-      <x:c r="F16" s="41" t="e">
+      <x:c r="F16" s="36" t="e">
         <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Quantitative_Summer_Analyst.pdf","Open PDF")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Balbec_Quantitative_Summer_Analyst.pdf, friendlyName=Open PDF</x:v>
       </x:c>
-      <x:c r="G16" s="43" t="str"/>
+      <x:c r="G16" s="38" t="str"/>
       <x:c r="H16" s="2"/>
       <x:c r="I16" s="2"/>
       <x:c r="J16" s="2"/>
       <x:c r="K16" s="2"/>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="2"/>
-      <x:c r="B17" s="2"/>
-      <x:c r="C17" s="2"/>
-      <x:c r="D17" s="2"/>
-      <x:c r="E17" s="2"/>
-      <x:c r="F17" s="2"/>
-      <x:c r="G17" s="2"/>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="35" t="str">
+        <x:v>Millennium Management</x:v>
+      </x:c>
+      <x:c r="B17" s="36" t="str">
+        <x:v>2027 Quantitative Researcher Intern, New York</x:v>
+      </x:c>
+      <x:c r="C17" s="37" t="n">
+        <x:v>46263</x:v>
+      </x:c>
+      <x:c r="D17" s="36" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E17" s="36" t="str">
+        <x:v>Workday receipt and candidacy update</x:v>
+      </x:c>
+      <x:c r="F17" s="36" t="str">
+        <x:v>Not captured</x:v>
+      </x:c>
+      <x:c r="G17" s="38" t="str">
+        <x:v>Application date comes from the employer receipt; later employer update states rejection.</x:v>
+      </x:c>
       <x:c r="H17" s="2"/>
       <x:c r="I17" s="2"/>
       <x:c r="J17" s="2"/>
       <x:c r="K17" s="2"/>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="2"/>
-      <x:c r="B18" s="2"/>
-      <x:c r="C18" s="2"/>
-      <x:c r="D18" s="2"/>
-      <x:c r="E18" s="2"/>
-      <x:c r="F18" s="2"/>
-      <x:c r="G18" s="2"/>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="35" t="str">
+        <x:v>Millennium Management</x:v>
+      </x:c>
+      <x:c r="B18" s="36" t="str">
+        <x:v>2027 Quantitative Developer Intern, New York</x:v>
+      </x:c>
+      <x:c r="C18" s="37" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="D18" s="36" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E18" s="36" t="str">
+        <x:v>Workday receipt and candidacy update</x:v>
+      </x:c>
+      <x:c r="F18" s="36" t="str">
+        <x:v>Not captured</x:v>
+      </x:c>
+      <x:c r="G18" s="38" t="str">
+        <x:v>Application date comes from the employer receipt; later employer update states rejection.</x:v>
+      </x:c>
       <x:c r="H18" s="2"/>
       <x:c r="I18" s="2"/>
       <x:c r="J18" s="2"/>
       <x:c r="K18" s="2"/>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="2"/>
-      <x:c r="B19" s="2"/>
-      <x:c r="C19" s="2"/>
-      <x:c r="D19" s="2"/>
-      <x:c r="E19" s="2"/>
-      <x:c r="F19" s="2"/>
-      <x:c r="G19" s="2"/>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="35" t="str">
+        <x:v>D. E. Shaw</x:v>
+      </x:c>
+      <x:c r="B19" s="36" t="str">
+        <x:v>Quantitative Analyst Intern, New York, Summer 2027</x:v>
+      </x:c>
+      <x:c r="C19" s="37" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="D19" s="36" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E19" s="36" t="str">
+        <x:v>Application receipt and employer update</x:v>
+      </x:c>
+      <x:c r="F19" s="36" t="e">
+        <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.DE_Shaw_Quantitative_Analyst_Intern.pdf","Open PDF")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.DE_Shaw_Quantitative_Analyst_Intern.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
+      <x:c r="G19" s="38" t="str"/>
       <x:c r="H19" s="2"/>
       <x:c r="I19" s="2"/>
       <x:c r="J19" s="2"/>
       <x:c r="K19" s="2"/>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="2"/>
-      <x:c r="B20" s="2"/>
-      <x:c r="C20" s="2"/>
-      <x:c r="D20" s="2"/>
-      <x:c r="E20" s="2"/>
-      <x:c r="F20" s="2"/>
-      <x:c r="G20" s="2"/>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="35" t="str">
+        <x:v>Jane Street</x:v>
+      </x:c>
+      <x:c r="B20" s="36" t="str">
+        <x:v>Role not specified in employer email</x:v>
+      </x:c>
+      <x:c r="C20" s="37" t="n">
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="D20" s="36" t="str">
+        <x:v>Rejected</x:v>
+      </x:c>
+      <x:c r="E20" s="36" t="str">
+        <x:v>Receipt and employer update</x:v>
+      </x:c>
+      <x:c r="F20" s="36" t="e">
+        <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Jane_Street_Quantitative_Researcher_Intern.pdf","Open PDF")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Jane_Street_Quantitative_Researcher_Intern.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
+      <x:c r="G20" s="38" t="str">
+        <x:v>Employer confirmation did not name the role; the linked PDF is the locally retained Jane Street tailored resume.</x:v>
+      </x:c>
       <x:c r="H20" s="2"/>
       <x:c r="I20" s="2"/>
       <x:c r="J20" s="2"/>
       <x:c r="K20" s="2"/>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
-      <x:c r="D21" s="2"/>
-      <x:c r="E21" s="2"/>
-      <x:c r="F21" s="2"/>
-      <x:c r="G21" s="2"/>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="35" t="str">
+        <x:v>Ridgeline</x:v>
+      </x:c>
+      <x:c r="B21" s="36" t="str">
+        <x:v>Software Engineer Intern, Summer 2027 (Cornell)</x:v>
+      </x:c>
+      <x:c r="C21" s="37" t="n">
+        <x:v>46283</x:v>
+      </x:c>
+      <x:c r="D21" s="36" t="str">
+        <x:v>Received / under review</x:v>
+      </x:c>
+      <x:c r="E21" s="36" t="str">
+        <x:v>Greenhouse confirmation email</x:v>
+      </x:c>
+      <x:c r="F21" s="36" t="str">
+        <x:v>Not captured</x:v>
+      </x:c>
+      <x:c r="G21" s="38" t="str">
+        <x:v>No role-specific PDF found locally.</x:v>
+      </x:c>
       <x:c r="H21" s="2"/>
       <x:c r="I21" s="2"/>
       <x:c r="J21" s="2"/>
       <x:c r="K21" s="2"/>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="2"/>
-      <x:c r="B22" s="2"/>
-      <x:c r="C22" s="2"/>
-      <x:c r="D22" s="2"/>
-      <x:c r="E22" s="2"/>
-      <x:c r="F22" s="2"/>
-      <x:c r="G22" s="2"/>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="35" t="str">
+        <x:v>Susquehanna</x:v>
+      </x:c>
+      <x:c r="B22" s="36" t="str">
+        <x:v>Quantitative Research position</x:v>
+      </x:c>
+      <x:c r="C22" s="37" t="n">
+        <x:v>46274</x:v>
+      </x:c>
+      <x:c r="D22" s="36" t="str">
+        <x:v>OA received</x:v>
+      </x:c>
+      <x:c r="E22" s="36" t="str">
+        <x:v>Recruiting and Mettl assessment invitations</x:v>
+      </x:c>
+      <x:c r="F22" s="36" t="e">
+        <x:f>HYPERLINK("https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Susquehanna_Quantitative_Research_Intern.pdf","Open PDF")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=https://github.com/xujingxiang19883/job-applications-dashboard-2026/blob/main/resumes/Xu.Jingxiang.Susquehanna_Quantitative_Research_Intern.pdf, friendlyName=Open PDF</x:v>
+      </x:c>
+      <x:c r="G22" s="38" t="str">
+        <x:v>Assessment invitation confirms both open positions; the date shown is the invitation date.</x:v>
+      </x:c>
       <x:c r="H22" s="2"/>
       <x:c r="I22" s="2"/>
       <x:c r="J22" s="2"/>
       <x:c r="K22" s="2"/>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="2"/>
-      <x:c r="B23" s="2"/>
-      <x:c r="C23" s="2"/>
-      <x:c r="D23" s="2"/>
-      <x:c r="E23" s="2"/>
-      <x:c r="F23" s="2"/>
-      <x:c r="G23" s="2"/>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="A23" s="39" t="str">
+        <x:v>Susquehanna</x:v>
+      </x:c>
+      <x:c r="B23" s="40" t="str">
+        <x:v>Quantitative Systematic Trading position</x:v>
+      </x:c>
+      <x:c r="C23" s="41" t="n">
+        <x:v>46274</x:v>
+      </x:c>
+      <x:c r="D23" s="40" t="str">
+        <x:v>OA received</x:v>
+      </x:c>
+      <x:c r="E23" s="40" t="str">
+        <x:v>Recruiting and Mettl assessment invitations</x:v>
+      </x:c>
+      <x:c r="F23" s="40" t="str">
+        <x:v>Not captured</x:v>
+      </x:c>
+      <x:c r="G23" s="42" t="str">
+        <x:v>Assessment invitation confirms both open positions; the date shown is the invitation date.</x:v>
+      </x:c>
       <x:c r="H23" s="2"/>
       <x:c r="I23" s="2"/>
       <x:c r="J23" s="2"/>
@@ -3183,7 +3408,7 @@
     <x:mergeCell ref="A2:G2"/>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D6:D16">
+  <x:conditionalFormatting sqref="D6:D23">
     <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Assessment"/>
     <x:cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="received"/>
     <x:cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="Submitted"/>

</xml_diff>